<commit_message>
Push full project to CRDTransport/vanchuyen
</commit_message>
<xml_diff>
--- a/Img/Bảng_giá_US.xlsx
+++ b/Img/Bảng_giá_US.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\My Computer\Documents\Zalo Received Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jang\Downloads\vanchuyen\Img\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB603244-10BC-4000-8C25-A6A5A4901945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FCA5274-307F-422C-AC54-AC47E345E726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bảng giá" sheetId="1" r:id="rId1"/>
@@ -78,9 +78,6 @@
     <t>3. Hàng dễ vỡ như Gốm sứ, thủy tinh, kính…: Bảo hiểm mất, thất lạc nhưng không bảo hiểm hàng vỡ nếu đóng hàng không đúng quy cách với hàng dễ vỡ</t>
   </si>
   <si>
-    <t>3. Nhóm hàng điện tử: Loa đài, Ampli, điện thoại, laptop, nước hoa…</t>
-  </si>
-  <si>
     <t>Có phụ thu tùy loại</t>
   </si>
   <si>
@@ -119,6 +116,9 @@
   </si>
   <si>
     <t xml:space="preserve"> - Kho US: 9-15 ngày</t>
+  </si>
+  <si>
+    <t>3. Nhóm hàng mỹ phẩm, thực phẩm chức năng, điện tử: Loa đài, Ampli, điện thoại, laptop, nước hoa…</t>
   </si>
 </sst>
 </file>
@@ -445,164 +445,164 @@
   </cellStyleXfs>
   <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="2" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="2" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="37" fontId="2" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="2" fillId="0" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="2" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="2" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="2" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="37" fontId="2" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="37" fontId="2" fillId="0" borderId="12" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="2" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="37" fontId="2" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="2" fillId="0" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="2" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="2" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="2" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="2" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -926,235 +926,235 @@
   <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="63.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="41.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="63.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="32"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="32"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="13"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="32"/>
+      <c r="A3" s="11"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="13"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="32"/>
+      <c r="A4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="13"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="32"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="13"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="33"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="16"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="8" t="s">
+      <c r="B7" s="44"/>
+      <c r="C7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="36" t="s">
+      <c r="D7" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="37"/>
+      <c r="E7" s="18"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="9"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="34"/>
-      <c r="E8" s="38"/>
+      <c r="A8" s="45"/>
+      <c r="B8" s="46"/>
+      <c r="C8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="19"/>
+      <c r="E8" s="20"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="48"/>
+      <c r="C9" s="5">
+        <v>245000</v>
+      </c>
+      <c r="D9" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="14">
-        <v>235000</v>
-      </c>
-      <c r="D9" s="39" t="s">
+      <c r="E9" s="22"/>
+    </row>
+    <row r="10" spans="1:5" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="39" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="40"/>
+      <c r="C10" s="5">
+        <v>255000</v>
+      </c>
+      <c r="D10" s="49" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="50"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="42"/>
+      <c r="C11" s="51" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="52"/>
+      <c r="E11" s="53"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="9">
+        <v>380000</v>
+      </c>
+      <c r="D12" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="31"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="40"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="14">
-        <v>245000</v>
-      </c>
-      <c r="D10" s="41" t="s">
+      <c r="B13" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" s="9">
+        <v>500000</v>
+      </c>
+      <c r="D13" s="32"/>
+      <c r="E13" s="33"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="9">
+        <v>50000</v>
+      </c>
+      <c r="D14" s="32"/>
+      <c r="E14" s="33"/>
+    </row>
+    <row r="15" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="42"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="35" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="43"/>
-      <c r="E11" s="44"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="20" t="s">
+      <c r="B15" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="21">
-        <v>380000</v>
-      </c>
-      <c r="D12" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="46"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="20" t="s">
+      <c r="C15" s="9">
+        <v>100000</v>
+      </c>
+      <c r="D15" s="32"/>
+      <c r="E15" s="33"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="21">
-        <v>500000</v>
-      </c>
-      <c r="D13" s="47"/>
-      <c r="E13" s="48"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="C16" s="9">
+        <v>350000</v>
+      </c>
+      <c r="D16" s="32"/>
+      <c r="E16" s="33"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17" s="9">
+        <v>600000</v>
+      </c>
+      <c r="D17" s="32"/>
+      <c r="E17" s="33"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B18" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="21">
-        <v>50000</v>
-      </c>
-      <c r="D14" s="47"/>
-      <c r="E14" s="48"/>
-    </row>
-    <row r="15" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="20" t="s">
+      <c r="C18" s="9">
+        <v>900000</v>
+      </c>
+      <c r="D18" s="32"/>
+      <c r="E18" s="33"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="21">
-        <v>100000</v>
-      </c>
-      <c r="D15" s="47"/>
-      <c r="E15" s="48"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
-        <v>6</v>
-      </c>
-      <c r="B16" s="20" t="s">
+      <c r="C19" s="9">
+        <v>1000000</v>
+      </c>
+      <c r="D19" s="32"/>
+      <c r="E19" s="33"/>
+    </row>
+    <row r="20" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="21">
-        <v>350000</v>
-      </c>
-      <c r="D16" s="47"/>
-      <c r="E16" s="48"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="C17" s="21">
-        <v>600000</v>
-      </c>
-      <c r="D17" s="47"/>
-      <c r="E17" s="48"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" s="21">
-        <v>900000</v>
-      </c>
-      <c r="D18" s="47"/>
-      <c r="E18" s="48"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B19" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="C19" s="21">
-        <v>1000000</v>
-      </c>
-      <c r="D19" s="47"/>
-      <c r="E19" s="48"/>
-    </row>
-    <row r="20" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="49"/>
-      <c r="E20" s="50"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="35"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="24"/>
@@ -1164,15 +1164,15 @@
       <c r="E21" s="24"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="51" t="s">
+      <c r="A22" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="52"/>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="53"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
@@ -1184,52 +1184,54 @@
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="28" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="29"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="30"/>
+      <c r="A24" s="27" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="29"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="26" t="s">
+      <c r="A25" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="27" t="s">
+      <c r="A26" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
+      <c r="B26" s="26"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
+      <c r="B27" s="26"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="26" t="s">
+      <c r="A28" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="C11:E11"/>
     <mergeCell ref="A1:E6"/>
     <mergeCell ref="D7:E8"/>
     <mergeCell ref="D9:E9"/>
@@ -1246,8 +1248,6 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A7:B8"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="C11:E11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>